<commit_message>
Update model outputs 2026-08-15 11:16:21
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="32">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,34 +44,25 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
   </si>
   <si>
     <t xml:space="preserve">Provisional</t>
   </si>
   <si>
+    <t xml:space="preserve">Marvel Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
     <t xml:space="preserve">IKON Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Marvel Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
   </si>
   <si>
     <t xml:space="preserve">gold coast suns</t>
@@ -497,7 +488,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46247</v>
+        <v>46249</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -512,16 +503,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>28.4</v>
+        <v>-42</v>
       </c>
       <c r="G2" t="n">
-        <v>13.3</v>
+        <v>-25</v>
       </c>
       <c r="H2" t="n">
-        <v>30.9</v>
+        <v>-47.3</v>
       </c>
       <c r="I2" t="n">
-        <v>82.9</v>
+        <v>86.2</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -538,25 +529,25 @@
         <v>15</v>
       </c>
       <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="H3" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="I3" t="n">
+        <v>73.9</v>
+      </c>
+      <c r="J3" t="s">
         <v>16</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-47.5</v>
-      </c>
-      <c r="G3" t="n">
-        <v>-25</v>
-      </c>
-      <c r="H3" t="n">
-        <v>-51.8</v>
-      </c>
-      <c r="I3" t="n">
-        <v>86.2</v>
-      </c>
-      <c r="J3" t="s">
-        <v>17</v>
       </c>
     </row>
     <row r="4">
@@ -564,36 +555,36 @@
         <v>46249</v>
       </c>
       <c r="B4" t="s">
+        <v>17</v>
+      </c>
+      <c r="C4" t="s">
         <v>18</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>12</v>
+      </c>
+      <c r="F4" t="n">
+        <v>-7.8</v>
+      </c>
+      <c r="G4" t="n">
+        <v>19.2</v>
+      </c>
+      <c r="H4" t="n">
+        <v>-1.8</v>
+      </c>
+      <c r="I4" t="n">
+        <v>80.9</v>
+      </c>
+      <c r="J4" t="s">
         <v>19</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4" t="s">
-        <v>16</v>
-      </c>
-      <c r="F4" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="G4" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="H4" t="n">
-        <v>7.9</v>
-      </c>
-      <c r="I4" t="n">
-        <v>73.9</v>
-      </c>
-      <c r="J4" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46249</v>
+        <v>46250</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -602,22 +593,22 @@
         <v>21</v>
       </c>
       <c r="D5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>22.4</v>
+        <v>22.5</v>
       </c>
       <c r="G5" t="n">
-        <v>19.2</v>
+        <v>17.8</v>
       </c>
       <c r="H5" t="n">
-        <v>32.1</v>
+        <v>25.1</v>
       </c>
       <c r="I5" t="n">
-        <v>80.9</v>
+        <v>79.6</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -634,22 +625,22 @@
         <v>24</v>
       </c>
       <c r="D6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E6" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>41</v>
+        <v>1.7</v>
       </c>
       <c r="G6" t="n">
-        <v>17.8</v>
+        <v>-5.8</v>
       </c>
       <c r="H6" t="n">
-        <v>45.5</v>
+        <v>6.1</v>
       </c>
       <c r="I6" t="n">
-        <v>79.6</v>
+        <v>83.5</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -666,22 +657,22 @@
         <v>27</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E7" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>-20.8</v>
+        <v>-4.1</v>
       </c>
       <c r="G7" t="n">
-        <v>-5.8</v>
+        <v>2.6</v>
       </c>
       <c r="H7" t="n">
-        <v>-22.3</v>
+        <v>-0.4</v>
       </c>
       <c r="I7" t="n">
-        <v>83.5</v>
+        <v>87.5</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
@@ -698,57 +689,25 @@
         <v>30</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="E8" t="s">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>-8.6</v>
+        <v>6.2</v>
       </c>
       <c r="G8" t="n">
-        <v>2.6</v>
+        <v>8.8</v>
       </c>
       <c r="H8" t="n">
-        <v>-1.5</v>
+        <v>6.7</v>
       </c>
       <c r="I8" t="n">
-        <v>87.5</v>
+        <v>82.7</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46250</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>16</v>
-      </c>
-      <c r="E9" t="s">
-        <v>16</v>
-      </c>
-      <c r="F9" t="n">
-        <v>15.1</v>
-      </c>
-      <c r="G9" t="n">
-        <v>8.8</v>
-      </c>
-      <c r="H9" t="n">
-        <v>23.2</v>
-      </c>
-      <c r="I9" t="n">
-        <v>82.7</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-08-29 09:56:41
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -44,88 +44,88 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
     <t xml:space="preserve">western bulldogs</t>
   </si>
   <si>
+    <t xml:space="preserve">Previous</t>
+  </si>
+  <si>
+    <t xml:space="preserve">University of Tasmania Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">waalitj marawar</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Thomas Farms Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">C.ex Coffs International Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
+  </si>
+  <si>
+    <t xml:space="preserve">melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Casey Fields</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">People First Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Victoria Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cockburn ARC Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
     <t xml:space="preserve">richmond</t>
   </si>
   <si>
-    <t xml:space="preserve">Provisional</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mission Whitten Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">west coast eagles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mineral Resources Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GMHBA Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brighton Homes Arena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SCG</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casey Fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">IKON Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alberton Oval</t>
+    <t xml:space="preserve">TIO Stadium</t>
   </si>
 </sst>
 </file>
@@ -461,15 +461,15 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="17.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="22.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="32.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +506,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -521,16 +521,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-7.7</v>
+        <v>-61.6</v>
       </c>
       <c r="G2" t="n">
-        <v>-13</v>
+        <v>-19.9</v>
       </c>
       <c r="H2" t="n">
-        <v>-14.6</v>
+        <v>-69.4</v>
       </c>
       <c r="I2" t="n">
-        <v>76</v>
+        <v>80.4</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -538,7 +538,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -553,16 +553,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-3.9</v>
+        <v>-37.5</v>
       </c>
       <c r="G3" t="n">
-        <v>-16.8</v>
+        <v>-6.2</v>
       </c>
       <c r="H3" t="n">
-        <v>-1.8</v>
+        <v>-34.6</v>
       </c>
       <c r="I3" t="n">
-        <v>80.8</v>
+        <v>83</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -570,7 +570,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46256</v>
+        <v>46263</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -585,16 +585,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-13.6</v>
+        <v>-35.7</v>
       </c>
       <c r="G4" t="n">
-        <v>-3.7</v>
+        <v>-6.8</v>
       </c>
       <c r="H4" t="n">
-        <v>-17.8</v>
+        <v>-39.4</v>
       </c>
       <c r="I4" t="n">
-        <v>81.1</v>
+        <v>80.4</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -602,7 +602,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46256</v>
+        <v>46264</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -617,16 +617,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>24</v>
+        <v>16.2</v>
       </c>
       <c r="G5" t="n">
-        <v>11.2</v>
+        <v>13.6</v>
       </c>
       <c r="H5" t="n">
-        <v>26.9</v>
+        <v>14.6</v>
       </c>
       <c r="I5" t="n">
-        <v>87.1</v>
+        <v>96.5</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -634,7 +634,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -649,16 +649,16 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-19.6</v>
+        <v>-1.6</v>
       </c>
       <c r="G6" t="n">
-        <v>-10.5</v>
+        <v>-1.4</v>
       </c>
       <c r="H6" t="n">
-        <v>-21.9</v>
+        <v>-7.6</v>
       </c>
       <c r="I6" t="n">
-        <v>78.4</v>
+        <v>87.9</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
@@ -681,16 +681,16 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>12.3</v>
+        <v>7.3</v>
       </c>
       <c r="G7" t="n">
-        <v>4.3</v>
+        <v>13.9</v>
       </c>
       <c r="H7" t="n">
-        <v>14.3</v>
+        <v>1.4</v>
       </c>
       <c r="I7" t="n">
-        <v>71.3</v>
+        <v>87.1</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B8" t="s">
         <v>29</v>
@@ -713,16 +713,16 @@
         <v>12</v>
       </c>
       <c r="F8" t="n">
-        <v>-40.4</v>
+        <v>-5.7</v>
       </c>
       <c r="G8" t="n">
-        <v>-25.2</v>
+        <v>5.4</v>
       </c>
       <c r="H8" t="n">
-        <v>-44.8</v>
+        <v>-8.8</v>
       </c>
       <c r="I8" t="n">
-        <v>90.1</v>
+        <v>73.7</v>
       </c>
       <c r="J8" t="s">
         <v>31</v>
@@ -730,7 +730,7 @@
     </row>
     <row r="9">
       <c r="A9" s="1" t="n">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B9" t="s">
         <v>32</v>
@@ -745,16 +745,16 @@
         <v>12</v>
       </c>
       <c r="F9" t="n">
-        <v>7.4</v>
+        <v>-10.3</v>
       </c>
       <c r="G9" t="n">
-        <v>-3.5</v>
+        <v>4.6</v>
       </c>
       <c r="H9" t="n">
-        <v>4.2</v>
+        <v>-10.7</v>
       </c>
       <c r="I9" t="n">
-        <v>87.5</v>
+        <v>82.4</v>
       </c>
       <c r="J9" t="s">
         <v>34</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="n">
-        <v>46257</v>
+        <v>46264</v>
       </c>
       <c r="B10" t="s">
         <v>35</v>
@@ -777,16 +777,16 @@
         <v>12</v>
       </c>
       <c r="F10" t="n">
-        <v>-12.3</v>
+        <v>-12.6</v>
       </c>
       <c r="G10" t="n">
-        <v>-7.9</v>
+        <v>0.4</v>
       </c>
       <c r="H10" t="n">
-        <v>-12.9</v>
+        <v>-20.4</v>
       </c>
       <c r="I10" t="n">
-        <v>89.5</v>
+        <v>75.4</v>
       </c>
       <c r="J10" t="s">
         <v>37</v>

</xml_diff>

<commit_message>
Update model outputs 2026-08-30 14:39:14
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,40 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">western bulldogs</t>
+    <t xml:space="preserve">greater western sydney</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">University of Tasmania Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">adelaide crows</t>
-  </si>
-  <si>
-    <t xml:space="preserve">waalitj marawar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Thomas Farms Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">C.ex Coffs International Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
   </si>
   <si>
     <t xml:space="preserve">Corroboree Group Oval Manuka</t>
@@ -462,14 +435,14 @@
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
     <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="32.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="28.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -506,7 +479,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -521,16 +494,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>-61.6</v>
+        <v>16.2</v>
       </c>
       <c r="G2" t="n">
-        <v>-19.9</v>
+        <v>13.6</v>
       </c>
       <c r="H2" t="n">
-        <v>-69.4</v>
+        <v>14.6</v>
       </c>
       <c r="I2" t="n">
-        <v>80.4</v>
+        <v>96.5</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -538,7 +511,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -553,16 +526,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-37.5</v>
+        <v>-1.6</v>
       </c>
       <c r="G3" t="n">
-        <v>-6.2</v>
+        <v>-1.4</v>
       </c>
       <c r="H3" t="n">
-        <v>-34.6</v>
+        <v>-7.6</v>
       </c>
       <c r="I3" t="n">
-        <v>83</v>
+        <v>87.9</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -570,7 +543,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46263</v>
+        <v>46264</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -585,16 +558,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-35.7</v>
+        <v>7.3</v>
       </c>
       <c r="G4" t="n">
-        <v>-6.8</v>
+        <v>13.9</v>
       </c>
       <c r="H4" t="n">
-        <v>-39.4</v>
+        <v>1.4</v>
       </c>
       <c r="I4" t="n">
-        <v>80.4</v>
+        <v>87.1</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -617,16 +590,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>16.2</v>
+        <v>-5.7</v>
       </c>
       <c r="G5" t="n">
-        <v>13.6</v>
+        <v>5.4</v>
       </c>
       <c r="H5" t="n">
-        <v>14.6</v>
+        <v>-8.8</v>
       </c>
       <c r="I5" t="n">
-        <v>96.5</v>
+        <v>73.7</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -649,16 +622,16 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-1.6</v>
+        <v>-10.3</v>
       </c>
       <c r="G6" t="n">
-        <v>-1.4</v>
+        <v>4.6</v>
       </c>
       <c r="H6" t="n">
-        <v>-7.6</v>
+        <v>-10.7</v>
       </c>
       <c r="I6" t="n">
-        <v>87.9</v>
+        <v>82.4</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -681,115 +654,19 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>7.3</v>
+        <v>-12.6</v>
       </c>
       <c r="G7" t="n">
-        <v>13.9</v>
+        <v>0.4</v>
       </c>
       <c r="H7" t="n">
-        <v>1.4</v>
+        <v>-20.4</v>
       </c>
       <c r="I7" t="n">
-        <v>87.1</v>
+        <v>75.4</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-5.7</v>
-      </c>
-      <c r="G8" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-8.8</v>
-      </c>
-      <c r="I8" t="n">
-        <v>73.7</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-10.3</v>
-      </c>
-      <c r="G9" t="n">
-        <v>4.6</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-10.7</v>
-      </c>
-      <c r="I9" t="n">
-        <v>82.4</v>
-      </c>
-      <c r="J9" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46264</v>
-      </c>
-      <c r="B10" t="s">
-        <v>35</v>
-      </c>
-      <c r="C10" t="s">
-        <v>36</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="n">
-        <v>-12.6</v>
-      </c>
-      <c r="G10" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="H10" t="n">
-        <v>-20.4</v>
-      </c>
-      <c r="I10" t="n">
-        <v>75.4</v>
-      </c>
-      <c r="J10" t="s">
-        <v>37</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-09-01 20:22:48
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="29" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,61 +44,85 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
+    <t xml:space="preserve">western bulldogs</t>
+  </si>
+  <si>
+    <t xml:space="preserve">sydney swans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Previous</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mission Whitten Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">st kilda</t>
+  </si>
+  <si>
+    <t xml:space="preserve">north melbourne</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RSEA Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">port adelaide</t>
+  </si>
+  <si>
+    <t xml:space="preserve">gold coast suns</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alberton Oval</t>
+  </si>
+  <si>
+    <t xml:space="preserve">brisbane lions</t>
+  </si>
+  <si>
     <t xml:space="preserve">greater western sydney</t>
   </si>
   <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Corroboree Group Oval Manuka</t>
+    <t xml:space="preserve">Brighton Homes Arena</t>
+  </si>
+  <si>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IKON Park</t>
+  </si>
+  <si>
+    <t xml:space="preserve">hawthorn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">adelaide crows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kennedy Community Centre</t>
+  </si>
+  <si>
+    <t xml:space="preserve">geelong cats</t>
+  </si>
+  <si>
+    <t xml:space="preserve">essendon</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GMHBA Stadium</t>
+  </si>
+  <si>
+    <t xml:space="preserve">carlton</t>
+  </si>
+  <si>
+    <t xml:space="preserve">collingwood</t>
+  </si>
+  <si>
+    <t xml:space="preserve">waalitj marawar</t>
   </si>
   <si>
     <t xml:space="preserve">melbourne</t>
   </si>
   <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Casey Fields</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">geelong cats</t>
-  </si>
-  <si>
-    <t xml:space="preserve">People First Stadium</t>
-  </si>
-  <si>
-    <t xml:space="preserve">collingwood</t>
-  </si>
-  <si>
-    <t xml:space="preserve">hawthorn</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Victoria Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
-  </si>
-  <si>
-    <t xml:space="preserve">carlton</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cockburn ARC Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">essendon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">TIO Stadium</t>
+    <t xml:space="preserve">Mineral Resources Park</t>
   </si>
 </sst>
 </file>
@@ -434,15 +458,15 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="22.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
     <col min="7" max="7" width="24.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="26.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="15.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="28.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="24.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -479,7 +503,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46264</v>
+        <v>46270</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -494,16 +518,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>16.2</v>
+        <v>16.7</v>
       </c>
       <c r="G2" t="n">
-        <v>13.6</v>
+        <v>-6.5</v>
       </c>
       <c r="H2" t="n">
-        <v>14.6</v>
+        <v>20.5</v>
       </c>
       <c r="I2" t="n">
-        <v>96.5</v>
+        <v>79.3</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -511,7 +535,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46264</v>
+        <v>46270</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -526,16 +550,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>-1.6</v>
+        <v>50</v>
       </c>
       <c r="G3" t="n">
-        <v>-1.4</v>
+        <v>29.6</v>
       </c>
       <c r="H3" t="n">
-        <v>-7.6</v>
+        <v>48.2</v>
       </c>
       <c r="I3" t="n">
-        <v>87.9</v>
+        <v>81.4</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -543,7 +567,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46264</v>
+        <v>46270</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -558,16 +582,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>7.3</v>
+        <v>-10.1</v>
       </c>
       <c r="G4" t="n">
-        <v>13.9</v>
+        <v>-21.3</v>
       </c>
       <c r="H4" t="n">
-        <v>1.4</v>
+        <v>-7.3</v>
       </c>
       <c r="I4" t="n">
-        <v>87.1</v>
+        <v>94.8</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -575,7 +599,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46264</v>
+        <v>46270</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -590,16 +614,16 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>-5.7</v>
+        <v>-41.6</v>
       </c>
       <c r="G5" t="n">
-        <v>5.4</v>
+        <v>-25.7</v>
       </c>
       <c r="H5" t="n">
-        <v>-8.8</v>
+        <v>-43.7</v>
       </c>
       <c r="I5" t="n">
-        <v>73.7</v>
+        <v>89.4</v>
       </c>
       <c r="J5" t="s">
         <v>22</v>
@@ -607,7 +631,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46264</v>
+        <v>46271</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -622,16 +646,16 @@
         <v>12</v>
       </c>
       <c r="F6" t="n">
-        <v>-10.3</v>
+        <v>26.3</v>
       </c>
       <c r="G6" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
       <c r="H6" t="n">
-        <v>-10.7</v>
+        <v>35.1</v>
       </c>
       <c r="I6" t="n">
-        <v>82.4</v>
+        <v>75.6</v>
       </c>
       <c r="J6" t="s">
         <v>25</v>
@@ -639,7 +663,7 @@
     </row>
     <row r="7">
       <c r="A7" s="1" t="n">
-        <v>46264</v>
+        <v>46271</v>
       </c>
       <c r="B7" t="s">
         <v>26</v>
@@ -654,19 +678,115 @@
         <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>-12.6</v>
+        <v>12.5</v>
       </c>
       <c r="G7" t="n">
-        <v>0.4</v>
+        <v>3.9</v>
       </c>
       <c r="H7" t="n">
-        <v>-20.4</v>
+        <v>15.9</v>
       </c>
       <c r="I7" t="n">
-        <v>75.4</v>
+        <v>80.4</v>
       </c>
       <c r="J7" t="s">
         <v>28</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B8" t="s">
+        <v>29</v>
+      </c>
+      <c r="C8" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>12</v>
+      </c>
+      <c r="F8" t="n">
+        <v>-9.6</v>
+      </c>
+      <c r="G8" t="n">
+        <v>-8.3</v>
+      </c>
+      <c r="H8" t="n">
+        <v>-5.3</v>
+      </c>
+      <c r="I8" t="n">
+        <v>79.9</v>
+      </c>
+      <c r="J8" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>33</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>12</v>
+      </c>
+      <c r="F9" t="n">
+        <v>-20.8</v>
+      </c>
+      <c r="G9" t="n">
+        <v>-13.1</v>
+      </c>
+      <c r="H9" t="n">
+        <v>-25.3</v>
+      </c>
+      <c r="I9" t="n">
+        <v>80.8</v>
+      </c>
+      <c r="J9" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="n">
+        <v>46271</v>
+      </c>
+      <c r="B10" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" t="s">
+        <v>35</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>12</v>
+      </c>
+      <c r="F10" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H10" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="I10" t="n">
+        <v>86.1</v>
+      </c>
+      <c r="J10" t="s">
+        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update model outputs 2026-09-06 22:12:00
</commit_message>
<xml_diff>
--- a/files/AFLW_upcoming_projections.xlsx
+++ b/files/AFLW_upcoming_projections.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="25">
   <si>
     <t xml:space="preserve">Date</t>
   </si>
@@ -44,49 +44,13 @@
     <t xml:space="preserve">Venue</t>
   </si>
   <si>
-    <t xml:space="preserve">western bulldogs</t>
-  </si>
-  <si>
-    <t xml:space="preserve">sydney swans</t>
+    <t xml:space="preserve">richmond</t>
+  </si>
+  <si>
+    <t xml:space="preserve">fremantle</t>
   </si>
   <si>
     <t xml:space="preserve">Previous</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Mission Whitten Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">st kilda</t>
-  </si>
-  <si>
-    <t xml:space="preserve">north melbourne</t>
-  </si>
-  <si>
-    <t xml:space="preserve">RSEA Park</t>
-  </si>
-  <si>
-    <t xml:space="preserve">port adelaide</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gold coast suns</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alberton Oval</t>
-  </si>
-  <si>
-    <t xml:space="preserve">brisbane lions</t>
-  </si>
-  <si>
-    <t xml:space="preserve">greater western sydney</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Brighton Homes Arena</t>
-  </si>
-  <si>
-    <t xml:space="preserve">richmond</t>
-  </si>
-  <si>
-    <t xml:space="preserve">fremantle</t>
   </si>
   <si>
     <t xml:space="preserve">IKON Park</t>
@@ -458,8 +422,8 @@
   <sheetFormatPr defaultRowHeight="15.0" baseColWidth="10"/>
   <cols>
     <col min="1" max="1" width="5.71" hidden="0" customWidth="1"/>
-    <col min="2" max="2" width="16.71" hidden="0" customWidth="1"/>
-    <col min="3" max="3" width="22.71" hidden="0" customWidth="1"/>
+    <col min="2" max="2" width="15.71" hidden="0" customWidth="1"/>
+    <col min="3" max="3" width="14.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="14.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="14.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="19.71" hidden="0" customWidth="1"/>
@@ -503,7 +467,7 @@
     </row>
     <row r="2">
       <c r="A2" s="1" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="B2" t="s">
         <v>10</v>
@@ -518,16 +482,16 @@
         <v>12</v>
       </c>
       <c r="F2" t="n">
-        <v>16.7</v>
+        <v>26.3</v>
       </c>
       <c r="G2" t="n">
-        <v>-6.5</v>
+        <v>4.9</v>
       </c>
       <c r="H2" t="n">
-        <v>20.5</v>
+        <v>35.1</v>
       </c>
       <c r="I2" t="n">
-        <v>79.3</v>
+        <v>75.6</v>
       </c>
       <c r="J2" t="s">
         <v>13</v>
@@ -535,7 +499,7 @@
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="B3" t="s">
         <v>14</v>
@@ -550,16 +514,16 @@
         <v>12</v>
       </c>
       <c r="F3" t="n">
-        <v>50</v>
+        <v>12.5</v>
       </c>
       <c r="G3" t="n">
-        <v>29.6</v>
+        <v>3.9</v>
       </c>
       <c r="H3" t="n">
-        <v>48.2</v>
+        <v>15.9</v>
       </c>
       <c r="I3" t="n">
-        <v>81.4</v>
+        <v>80.4</v>
       </c>
       <c r="J3" t="s">
         <v>16</v>
@@ -567,7 +531,7 @@
     </row>
     <row r="4">
       <c r="A4" s="1" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="B4" t="s">
         <v>17</v>
@@ -582,16 +546,16 @@
         <v>12</v>
       </c>
       <c r="F4" t="n">
-        <v>-10.1</v>
+        <v>-9.6</v>
       </c>
       <c r="G4" t="n">
-        <v>-21.3</v>
+        <v>-8.3</v>
       </c>
       <c r="H4" t="n">
-        <v>-7.3</v>
+        <v>-5.3</v>
       </c>
       <c r="I4" t="n">
-        <v>94.8</v>
+        <v>79.9</v>
       </c>
       <c r="J4" t="s">
         <v>19</v>
@@ -599,7 +563,7 @@
     </row>
     <row r="5">
       <c r="A5" s="1" t="n">
-        <v>46270</v>
+        <v>46271</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -614,19 +578,19 @@
         <v>12</v>
       </c>
       <c r="F5" t="n">
-        <v>-41.6</v>
+        <v>-20.8</v>
       </c>
       <c r="G5" t="n">
-        <v>-25.7</v>
+        <v>-13.1</v>
       </c>
       <c r="H5" t="n">
-        <v>-43.7</v>
+        <v>-25.3</v>
       </c>
       <c r="I5" t="n">
-        <v>89.4</v>
+        <v>80.8</v>
       </c>
       <c r="J5" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
     </row>
     <row r="6">
@@ -634,159 +598,31 @@
         <v>46271</v>
       </c>
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>12</v>
+      </c>
+      <c r="F6" t="n">
+        <v>43.6</v>
+      </c>
+      <c r="G6" t="n">
+        <v>9.9</v>
+      </c>
+      <c r="H6" t="n">
+        <v>41.9</v>
+      </c>
+      <c r="I6" t="n">
+        <v>86.1</v>
+      </c>
+      <c r="J6" t="s">
         <v>24</v>
-      </c>
-      <c r="D6" t="s">
-        <v>12</v>
-      </c>
-      <c r="E6" t="s">
-        <v>12</v>
-      </c>
-      <c r="F6" t="n">
-        <v>26.3</v>
-      </c>
-      <c r="G6" t="n">
-        <v>4.9</v>
-      </c>
-      <c r="H6" t="n">
-        <v>35.1</v>
-      </c>
-      <c r="I6" t="n">
-        <v>75.6</v>
-      </c>
-      <c r="J6" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="1" t="n">
-        <v>46271</v>
-      </c>
-      <c r="B7" t="s">
-        <v>26</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>12</v>
-      </c>
-      <c r="E7" t="s">
-        <v>12</v>
-      </c>
-      <c r="F7" t="n">
-        <v>12.5</v>
-      </c>
-      <c r="G7" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="H7" t="n">
-        <v>15.9</v>
-      </c>
-      <c r="I7" t="n">
-        <v>80.4</v>
-      </c>
-      <c r="J7" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="1" t="n">
-        <v>46271</v>
-      </c>
-      <c r="B8" t="s">
-        <v>29</v>
-      </c>
-      <c r="C8" t="s">
-        <v>30</v>
-      </c>
-      <c r="D8" t="s">
-        <v>12</v>
-      </c>
-      <c r="E8" t="s">
-        <v>12</v>
-      </c>
-      <c r="F8" t="n">
-        <v>-9.6</v>
-      </c>
-      <c r="G8" t="n">
-        <v>-8.3</v>
-      </c>
-      <c r="H8" t="n">
-        <v>-5.3</v>
-      </c>
-      <c r="I8" t="n">
-        <v>79.9</v>
-      </c>
-      <c r="J8" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="n">
-        <v>46271</v>
-      </c>
-      <c r="B9" t="s">
-        <v>32</v>
-      </c>
-      <c r="C9" t="s">
-        <v>33</v>
-      </c>
-      <c r="D9" t="s">
-        <v>12</v>
-      </c>
-      <c r="E9" t="s">
-        <v>12</v>
-      </c>
-      <c r="F9" t="n">
-        <v>-20.8</v>
-      </c>
-      <c r="G9" t="n">
-        <v>-13.1</v>
-      </c>
-      <c r="H9" t="n">
-        <v>-25.3</v>
-      </c>
-      <c r="I9" t="n">
-        <v>80.8</v>
-      </c>
-      <c r="J9" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="1" t="n">
-        <v>46271</v>
-      </c>
-      <c r="B10" t="s">
-        <v>34</v>
-      </c>
-      <c r="C10" t="s">
-        <v>35</v>
-      </c>
-      <c r="D10" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" t="s">
-        <v>12</v>
-      </c>
-      <c r="F10" t="n">
-        <v>43.6</v>
-      </c>
-      <c r="G10" t="n">
-        <v>9.9</v>
-      </c>
-      <c r="H10" t="n">
-        <v>41.9</v>
-      </c>
-      <c r="I10" t="n">
-        <v>86.1</v>
-      </c>
-      <c r="J10" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>